<commit_message>
Add Excel-vs-PDF example to the README and match Excel chart defaults
- New samples/sales-report.xlsx with a screenshot of it in Microsoft Excel
  and the page excel2pdf renders, shown side by side in both READMEs.
- Chart defaults now follow what Excel draws for unstyled charts: data-label
  flags omitted from <c:dLbls> count as on, unstyled titles are bold at the
  chart text size, darker major gridlines, denser value-axis ticks, no white
  pie-slice borders, and pie percentages that add up to 100%.
- Sample charts set their data-label flags explicitly.
- Ignore Office lock files.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/charts.xlsx
+++ b/samples/charts.xlsx
@@ -319,7 +319,11 @@
           </val>
         </ser>
         <dLbls>
+          <showLegendKey val="0"/>
           <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="0"/>
         </dLbls>
         <gapWidth val="150"/>
         <axId val="10"/>
@@ -885,6 +889,10 @@
           </val>
         </ser>
         <dLbls>
+          <showLegendKey val="0"/>
+          <showVal val="0"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
           <showPercent val="1"/>
         </dLbls>
         <firstSliceAng val="0"/>

</xml_diff>

<commit_message>
Add Excel-vs-PDF example to the README and match Excel chart defaults (#1)
- New samples/sales-report.xlsx with a screenshot of it in Microsoft Excel
  and the page excel2pdf renders, shown side by side in both READMEs.
- Chart defaults now follow what Excel draws for unstyled charts: data-label
  flags omitted from <c:dLbls> count as on, unstyled titles are bold at the
  chart text size, darker major gridlines, denser value-axis ticks, no white
  pie-slice borders, and pie percentages that add up to 100%.
- Sample charts set their data-label flags explicitly.
- Ignore Office lock files.

Co-authored-by: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/charts.xlsx
+++ b/samples/charts.xlsx
@@ -319,7 +319,11 @@
           </val>
         </ser>
         <dLbls>
+          <showLegendKey val="0"/>
           <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
+          <showPercent val="0"/>
         </dLbls>
         <gapWidth val="150"/>
         <axId val="10"/>
@@ -885,6 +889,10 @@
           </val>
         </ser>
         <dLbls>
+          <showLegendKey val="0"/>
+          <showVal val="0"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
           <showPercent val="1"/>
         </dLbls>
         <firstSliceAng val="0"/>

</xml_diff>